<commit_message>
Need to fit rest and refit F1=3 lines
</commit_message>
<xml_diff>
--- a/894BackgroundCheck/Book1-100Width.xlsx
+++ b/894BackgroundCheck/Book1-100Width.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Wolfwalker\Documents\git\6s7p\894BackgroundCheck\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Diego\git\6s7p\894BackgroundCheck\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{591A6221-E641-4030-8929-833B9325C236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{408FD0B0-D988-4918-969F-8A12DD2BB005}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{7EC8DE92-3FC3-47D3-8B94-7582F045A6DE}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7EC8DE92-3FC3-47D3-8B94-7582F045A6DE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -903,7 +901,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2820,7 +2818,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -2828,6 +2825,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -4728,7 +4726,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -4736,6 +4733,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -6606,7 +6604,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -6614,6 +6611,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -7708,7 +7706,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -7716,6 +7713,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -8780,7 +8778,6 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
-    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -8788,6 +8785,7 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
+    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -11607,15 +11605,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>215900</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>539750</xdr:rowOff>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>187325</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>20</xdr:col>
-      <xdr:colOff>85725</xdr:colOff>
+      <xdr:colOff>47625</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
+      <xdr:rowOff>260350</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -11642,16 +11640,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>187325</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>263525</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>155575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>27</xdr:col>
-      <xdr:colOff>492125</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>69850</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>568325</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>136525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -11678,16 +11676,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>536574</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>368300</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>1050924</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>263525</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>44449</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>495300</xdr:rowOff>
+      <xdr:col>28</xdr:col>
+      <xdr:colOff>187324</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>390525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -12105,12 +12103,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1EA69FB3-EF00-4FCA-AC52-38EBDB1417E8}">
   <dimension ref="A1:S308"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="10" max="10" width="13.81640625" customWidth="1"/>
+    <col min="10" max="10" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="42.75">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -12148,7 +12146,7 @@
         <v>1.350139213627954</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" ht="42.75">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -12174,7 +12172,7 @@
         <v>1.34164808621162</v>
       </c>
       <c r="I2">
-        <f t="shared" ref="I2:I65" si="0">G2/H2</f>
+        <f>G2/H2</f>
         <v>4.9969669493333674E-3</v>
       </c>
       <c r="J2">
@@ -12186,7 +12184,7 @@
         <v>8.2414253775113071E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" ht="42.75">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -12212,11 +12210,15 @@
         <v>1.3378072444151301</v>
       </c>
       <c r="I3">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="I2:I65" si="0">G3/H3</f>
         <v>5.0012518152433546E-3</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="J3">
+        <f>J1-J2</f>
+        <v>1.6182171430964634E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="42.75">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -12246,7 +12248,7 @@
         <v>4.7770433366768677E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" ht="42.75">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -12276,7 +12278,7 @@
         <v>4.7905109826317143E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" ht="42.75">
       <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
@@ -12306,7 +12308,7 @@
         <v>4.7826951804041231E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" ht="42.75">
       <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
@@ -12336,7 +12338,7 @@
         <v>4.2391434815920283E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" ht="42.75">
       <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
@@ -12366,7 +12368,7 @@
         <v>4.0764188211235928E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" ht="42.75">
       <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
@@ -12396,7 +12398,7 @@
         <v>4.2869435611514392E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" ht="42.75">
       <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
@@ -12426,7 +12428,7 @@
         <v>4.6517370246778409E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" ht="42.75">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -12456,7 +12458,7 @@
         <v>4.1146858851064646E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" ht="42.75">
       <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
@@ -12486,7 +12488,7 @@
         <v>4.7493062915733384E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" ht="42.75">
       <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
@@ -12516,7 +12518,7 @@
         <v>4.2163702103224319E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" ht="42.75">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -12546,7 +12548,7 @@
         <v>3.6619869311992682E-3</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" ht="42.75">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -12576,7 +12578,7 @@
         <v>4.3975419135405059E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" ht="42.75">
       <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
@@ -12606,7 +12608,7 @@
         <v>3.6874396263607977E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:19" ht="42.75">
       <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
@@ -12636,7 +12638,7 @@
         <v>3.4839932128115543E-3</v>
       </c>
     </row>
-    <row r="18" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:19" ht="42.75">
       <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
@@ -12666,7 +12668,7 @@
         <v>3.9140897538079639E-3</v>
       </c>
     </row>
-    <row r="19" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:19" ht="42.75">
       <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
@@ -12696,7 +12698,7 @@
         <v>3.1168917514904798E-3</v>
       </c>
     </row>
-    <row r="20" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:19" ht="42.75">
       <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
@@ -12726,7 +12728,7 @@
         <v>3.9679149715213333E-3</v>
       </c>
     </row>
-    <row r="21" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:19" ht="42.75">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -12756,7 +12758,7 @@
         <v>3.7851461918386423E-3</v>
       </c>
     </row>
-    <row r="22" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:19" ht="42.75">
       <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
@@ -12789,7 +12791,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="23" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:19" ht="42.75">
       <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
@@ -12819,7 +12821,7 @@
         <v>3.5271693280876622E-3</v>
       </c>
     </row>
-    <row r="24" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:19" ht="42.75">
       <c r="K24" s="1" t="s">
         <v>23</v>
       </c>
@@ -12845,11 +12847,11 @@
         <v>1.33333371460048</v>
       </c>
       <c r="S24">
-        <f>Q24/R24</f>
+        <f t="shared" ref="S24:S41" si="1">Q24/R24</f>
         <v>5.7995650151637483E-3</v>
       </c>
     </row>
-    <row r="25" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:19" ht="42.75">
       <c r="K25" s="1" t="s">
         <v>24</v>
       </c>
@@ -12875,11 +12877,11 @@
         <v>1.3374516314435101</v>
       </c>
       <c r="S25">
-        <f>Q25/R25</f>
+        <f t="shared" si="1"/>
         <v>5.7582120815396157E-3</v>
       </c>
     </row>
-    <row r="26" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:19" ht="42.75">
       <c r="K26" s="1" t="s">
         <v>25</v>
       </c>
@@ -12905,11 +12907,11 @@
         <v>1.33206068392977</v>
       </c>
       <c r="S26">
-        <f>Q26/R26</f>
+        <f t="shared" si="1"/>
         <v>6.2183891187897614E-3</v>
       </c>
     </row>
-    <row r="27" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:19" ht="42.75">
       <c r="K27" s="1" t="s">
         <v>26</v>
       </c>
@@ -12935,11 +12937,11 @@
         <v>1.34562637161871</v>
       </c>
       <c r="S27">
-        <f>Q27/R27</f>
+        <f t="shared" si="1"/>
         <v>4.5757314508261954E-3</v>
       </c>
     </row>
-    <row r="28" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:19" ht="42.75">
       <c r="K28" s="1" t="s">
         <v>27</v>
       </c>
@@ -12965,11 +12967,11 @@
         <v>1.3415348879250499</v>
       </c>
       <c r="S28">
-        <f>Q28/R28</f>
+        <f t="shared" si="1"/>
         <v>4.8903765480427996E-3</v>
       </c>
     </row>
-    <row r="29" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:19" ht="42.75">
       <c r="K29" s="1" t="s">
         <v>28</v>
       </c>
@@ -12995,11 +12997,11 @@
         <v>1.34152540831514</v>
       </c>
       <c r="S29">
-        <f>Q29/R29</f>
+        <f t="shared" si="1"/>
         <v>5.0524736858068089E-3</v>
       </c>
     </row>
-    <row r="30" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:19" ht="42.75">
       <c r="K30" s="1" t="s">
         <v>29</v>
       </c>
@@ -13025,11 +13027,11 @@
         <v>1.3369010809641599</v>
       </c>
       <c r="S30">
-        <f>Q30/R30</f>
+        <f t="shared" si="1"/>
         <v>4.8543011135982082E-3</v>
       </c>
     </row>
-    <row r="31" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:19" ht="42.75">
       <c r="K31" s="1" t="s">
         <v>30</v>
       </c>
@@ -13055,11 +13057,11 @@
         <v>1.3403863508604199</v>
       </c>
       <c r="S31">
-        <f>Q31/R31</f>
+        <f t="shared" si="1"/>
         <v>4.7579098955948477E-3</v>
       </c>
     </row>
-    <row r="32" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:19" ht="42.75">
       <c r="K32" s="1" t="s">
         <v>31</v>
       </c>
@@ -13085,11 +13087,11 @@
         <v>1.33794498958323</v>
       </c>
       <c r="S32">
-        <f>Q32/R32</f>
+        <f t="shared" si="1"/>
         <v>4.8320936047426145E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:19" ht="42.75">
       <c r="K33" s="1" t="s">
         <v>32</v>
       </c>
@@ -13115,11 +13117,11 @@
         <v>1.34257705865433</v>
       </c>
       <c r="S33">
-        <f>Q33/R33</f>
+        <f t="shared" si="1"/>
         <v>4.7970368463524831E-3</v>
       </c>
     </row>
-    <row r="34" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:19" ht="42.75">
       <c r="K34" s="1" t="s">
         <v>33</v>
       </c>
@@ -13145,11 +13147,11 @@
         <v>1.33982159216228</v>
       </c>
       <c r="S34">
-        <f>Q34/R34</f>
+        <f t="shared" si="1"/>
         <v>5.1637368424376825E-3</v>
       </c>
     </row>
-    <row r="35" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:19" ht="42.75">
       <c r="K35" s="1" t="s">
         <v>34</v>
       </c>
@@ -13175,11 +13177,11 @@
         <v>1.3392027606441499</v>
       </c>
       <c r="S35">
-        <f>Q35/R35</f>
+        <f t="shared" si="1"/>
         <v>5.319506939047953E-3</v>
       </c>
     </row>
-    <row r="36" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:19" ht="42.75">
       <c r="K36" s="1" t="s">
         <v>35</v>
       </c>
@@ -13205,11 +13207,11 @@
         <v>1.3380723735179101</v>
       </c>
       <c r="S36">
-        <f>Q36/R36</f>
+        <f t="shared" si="1"/>
         <v>5.3220591521841113E-3</v>
       </c>
     </row>
-    <row r="37" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:19" ht="42.75">
       <c r="K37" s="1" t="s">
         <v>36</v>
       </c>
@@ -13235,11 +13237,11 @@
         <v>1.3337388266685699</v>
       </c>
       <c r="S37">
-        <f>Q37/R37</f>
+        <f t="shared" si="1"/>
         <v>5.3999622509945796E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:19" ht="42.75">
       <c r="K38" s="1" t="s">
         <v>37</v>
       </c>
@@ -13265,11 +13267,11 @@
         <v>1.3333263681838099</v>
       </c>
       <c r="S38">
-        <f>Q38/R38</f>
+        <f t="shared" si="1"/>
         <v>5.6482487006513813E-3</v>
       </c>
     </row>
-    <row r="39" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:19" ht="42.75">
       <c r="K39" s="1" t="s">
         <v>38</v>
       </c>
@@ -13295,11 +13297,11 @@
         <v>1.33088677630543</v>
       </c>
       <c r="S39">
-        <f>Q39/R39</f>
+        <f t="shared" si="1"/>
         <v>4.9210794626922153E-3</v>
       </c>
     </row>
-    <row r="40" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:19" ht="42.75">
       <c r="K40" s="1" t="s">
         <v>39</v>
       </c>
@@ -13325,11 +13327,11 @@
         <v>1.34545483379652</v>
       </c>
       <c r="S40">
-        <f>Q40/R40</f>
+        <f t="shared" si="1"/>
         <v>4.7749570386006867E-3</v>
       </c>
     </row>
-    <row r="41" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:19" ht="42.75">
       <c r="K41" s="1" t="s">
         <v>40</v>
       </c>
@@ -13355,11 +13357,11 @@
         <v>1.3394005096252599</v>
       </c>
       <c r="S41">
-        <f>Q41/R41</f>
+        <f t="shared" si="1"/>
         <v>5.2917666381611782E-3</v>
       </c>
     </row>
-    <row r="42" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:19" ht="42.75">
       <c r="A42" s="1" t="s">
         <v>41</v>
       </c>
@@ -13389,7 +13391,7 @@
         <v>3.2673998822558398E-3</v>
       </c>
     </row>
-    <row r="43" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:19" ht="42.75">
       <c r="A43" s="1" t="s">
         <v>42</v>
       </c>
@@ -13419,7 +13421,7 @@
         <v>3.4521597748427145E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:19" ht="42.75">
       <c r="A44" s="1" t="s">
         <v>43</v>
       </c>
@@ -13449,7 +13451,7 @@
         <v>3.5510546741122635E-3</v>
       </c>
     </row>
-    <row r="45" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:19" ht="42.75">
       <c r="A45" s="1" t="s">
         <v>44</v>
       </c>
@@ -13479,7 +13481,7 @@
         <v>3.7821901415360883E-3</v>
       </c>
     </row>
-    <row r="46" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:19" ht="42.75">
       <c r="A46" s="1" t="s">
         <v>45</v>
       </c>
@@ -13509,7 +13511,7 @@
         <v>3.3262047871142832E-3</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:19" ht="42.75">
       <c r="A47" s="1" t="s">
         <v>46</v>
       </c>
@@ -13539,7 +13541,7 @@
         <v>3.2594016271542091E-3</v>
       </c>
     </row>
-    <row r="48" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:19" ht="42.75">
       <c r="A48" s="1" t="s">
         <v>47</v>
       </c>
@@ -13569,7 +13571,7 @@
         <v>3.1391422467399715E-3</v>
       </c>
     </row>
-    <row r="49" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9" ht="42.75">
       <c r="A49" s="1" t="s">
         <v>48</v>
       </c>
@@ -13599,7 +13601,7 @@
         <v>3.6206536453635869E-3</v>
       </c>
     </row>
-    <row r="50" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9" ht="42.75">
       <c r="A50" s="1" t="s">
         <v>49</v>
       </c>
@@ -13629,7 +13631,7 @@
         <v>3.4591104957257244E-3</v>
       </c>
     </row>
-    <row r="51" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9" ht="42.75">
       <c r="A51" s="1" t="s">
         <v>50</v>
       </c>
@@ -13659,7 +13661,7 @@
         <v>3.3545536111597193E-3</v>
       </c>
     </row>
-    <row r="52" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9" ht="42.75">
       <c r="A52" s="1" t="s">
         <v>51</v>
       </c>
@@ -13689,7 +13691,7 @@
         <v>3.181786724799348E-3</v>
       </c>
     </row>
-    <row r="53" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9" ht="42.75">
       <c r="A53" s="1" t="s">
         <v>52</v>
       </c>
@@ -13719,7 +13721,7 @@
         <v>3.4587434481864309E-3</v>
       </c>
     </row>
-    <row r="54" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9" ht="42.75">
       <c r="A54" s="1" t="s">
         <v>53</v>
       </c>
@@ -13749,7 +13751,7 @@
         <v>3.7911255385899242E-3</v>
       </c>
     </row>
-    <row r="55" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9" ht="42.75">
       <c r="A55" s="1" t="s">
         <v>54</v>
       </c>
@@ -13779,7 +13781,7 @@
         <v>3.8176020275235921E-3</v>
       </c>
     </row>
-    <row r="56" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9" ht="42.75">
       <c r="A56" s="1" t="s">
         <v>55</v>
       </c>
@@ -13809,7 +13811,7 @@
         <v>3.9075874052642628E-3</v>
       </c>
     </row>
-    <row r="57" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9" ht="42.75">
       <c r="A57" s="1" t="s">
         <v>56</v>
       </c>
@@ -13839,7 +13841,7 @@
         <v>3.3188528548926616E-3</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9" ht="42.75">
       <c r="A58" s="1" t="s">
         <v>57</v>
       </c>
@@ -13869,7 +13871,7 @@
         <v>3.7997804788342583E-3</v>
       </c>
     </row>
-    <row r="59" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9" ht="42.75">
       <c r="A59" s="1" t="s">
         <v>58</v>
       </c>
@@ -13899,7 +13901,7 @@
         <v>3.4228474625871913E-3</v>
       </c>
     </row>
-    <row r="60" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:9" ht="42.75">
       <c r="A60" s="1" t="s">
         <v>59</v>
       </c>
@@ -13929,7 +13931,7 @@
         <v>3.54549642210287E-3</v>
       </c>
     </row>
-    <row r="61" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9" ht="42.75">
       <c r="A61" s="1" t="s">
         <v>60</v>
       </c>
@@ -13959,7 +13961,7 @@
         <v>3.5191636934843893E-3</v>
       </c>
     </row>
-    <row r="62" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9" ht="42.75">
       <c r="A62" s="1" t="s">
         <v>61</v>
       </c>
@@ -13989,7 +13991,7 @@
         <v>3.9153884006626147E-3</v>
       </c>
     </row>
-    <row r="63" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9" ht="42.75">
       <c r="A63" s="1" t="s">
         <v>62</v>
       </c>
@@ -14019,7 +14021,7 @@
         <v>3.9268844907303369E-3</v>
       </c>
     </row>
-    <row r="64" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9" ht="42.75">
       <c r="A64" s="1" t="s">
         <v>63</v>
       </c>
@@ -14049,7 +14051,7 @@
         <v>3.6530086632902501E-3</v>
       </c>
     </row>
-    <row r="65" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9" ht="42.75">
       <c r="A65" s="1" t="s">
         <v>64</v>
       </c>
@@ -14079,7 +14081,7 @@
         <v>4.0363804021874535E-3</v>
       </c>
     </row>
-    <row r="66" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9" ht="42.75">
       <c r="A66" s="1" t="s">
         <v>65</v>
       </c>
@@ -14105,11 +14107,11 @@
         <v>1.3452187077625299</v>
       </c>
       <c r="I66">
-        <f t="shared" ref="I66:I129" si="1">G66/H66</f>
+        <f t="shared" ref="I66:I129" si="2">G66/H66</f>
         <v>3.3582556033914116E-3</v>
       </c>
     </row>
-    <row r="67" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9" ht="42.75">
       <c r="A67" s="1" t="s">
         <v>66</v>
       </c>
@@ -14135,11 +14137,11 @@
         <v>1.34102844485261</v>
       </c>
       <c r="I67">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.0774760019920003E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9" ht="42.75">
       <c r="A68" s="1" t="s">
         <v>67</v>
       </c>
@@ -14165,11 +14167,11 @@
         <v>1.34153107565063</v>
       </c>
       <c r="I68">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.6711027534851851E-3</v>
       </c>
     </row>
-    <row r="69" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9" ht="42.75">
       <c r="A69" s="1" t="s">
         <v>68</v>
       </c>
@@ -14195,11 +14197,11 @@
         <v>1.3396472723782</v>
       </c>
       <c r="I69">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.767828018950101E-3</v>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9" ht="42.75">
       <c r="A70" s="1" t="s">
         <v>69</v>
       </c>
@@ -14225,11 +14227,11 @@
         <v>1.3376664579302999</v>
       </c>
       <c r="I70">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.9209983734223635E-3</v>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9" ht="42.75">
       <c r="A71" s="1" t="s">
         <v>70</v>
       </c>
@@ -14255,11 +14257,11 @@
         <v>1.3406072827544699</v>
       </c>
       <c r="I71">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.1195790476980573E-3</v>
       </c>
     </row>
-    <row r="72" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9" ht="42.75">
       <c r="A72" s="1" t="s">
         <v>71</v>
       </c>
@@ -14285,11 +14287,11 @@
         <v>1.34180375058167</v>
       </c>
       <c r="I72">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.1234959899091993E-3</v>
       </c>
     </row>
-    <row r="73" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9" ht="42.75">
       <c r="A73" s="1" t="s">
         <v>72</v>
       </c>
@@ -14315,11 +14317,11 @@
         <v>1.34195073786524</v>
       </c>
       <c r="I73">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>4.1053760487338919E-3</v>
       </c>
     </row>
-    <row r="74" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9" ht="42.75">
       <c r="A74" s="1" t="s">
         <v>73</v>
       </c>
@@ -14345,11 +14347,11 @@
         <v>1.34135248482172</v>
       </c>
       <c r="I74">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.7518690055516495E-3</v>
       </c>
     </row>
-    <row r="75" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:9" ht="42.75">
       <c r="A75" s="1" t="s">
         <v>74</v>
       </c>
@@ -14375,11 +14377,11 @@
         <v>1.3411690653574699</v>
       </c>
       <c r="I75">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.7332014700790636E-3</v>
       </c>
     </row>
-    <row r="76" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:9" ht="42.75">
       <c r="A76" s="1" t="s">
         <v>75</v>
       </c>
@@ -14405,11 +14407,11 @@
         <v>1.3554184123120201</v>
       </c>
       <c r="I76">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.6850332045312481E-3</v>
       </c>
     </row>
-    <row r="77" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:9" ht="42.75">
       <c r="A77" s="1" t="s">
         <v>76</v>
       </c>
@@ -14435,11 +14437,11 @@
         <v>1.3542746774865599</v>
       </c>
       <c r="I77">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.0131139914129101E-3</v>
       </c>
     </row>
-    <row r="78" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:9" ht="42.75">
       <c r="A78" s="1" t="s">
         <v>77</v>
       </c>
@@ -14465,11 +14467,11 @@
         <v>1.35543471478572</v>
       </c>
       <c r="I78">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5095703774195284E-3</v>
       </c>
     </row>
-    <row r="79" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:9" ht="42.75">
       <c r="A79" s="1" t="s">
         <v>78</v>
       </c>
@@ -14495,11 +14497,11 @@
         <v>1.3481041697221401</v>
       </c>
       <c r="I79">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5416101466238412E-3</v>
       </c>
     </row>
-    <row r="80" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:9" ht="42.75">
       <c r="A80" s="1" t="s">
         <v>79</v>
       </c>
@@ -14525,11 +14527,11 @@
         <v>1.3499704272545601</v>
       </c>
       <c r="I80">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.4117416002638011E-3</v>
       </c>
     </row>
-    <row r="81" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9" ht="42.75">
       <c r="A81" s="1" t="s">
         <v>80</v>
       </c>
@@ -14555,11 +14557,11 @@
         <v>1.34003488917312</v>
       </c>
       <c r="I81">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5044123117072634E-3</v>
       </c>
     </row>
-    <row r="82" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9" ht="42.75">
       <c r="A82" s="1" t="s">
         <v>81</v>
       </c>
@@ -14585,11 +14587,11 @@
         <v>1.36549010822499</v>
       </c>
       <c r="I82">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.7398021514035841E-3</v>
       </c>
     </row>
-    <row r="83" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9" ht="42.75">
       <c r="A83" s="1" t="s">
         <v>82</v>
       </c>
@@ -14615,11 +14617,11 @@
         <v>1.3533809921025</v>
       </c>
       <c r="I83">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.7689265876288255E-3</v>
       </c>
     </row>
-    <row r="84" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9" ht="42.75">
       <c r="A84" s="1" t="s">
         <v>83</v>
       </c>
@@ -14645,11 +14647,11 @@
         <v>1.35944617560065</v>
       </c>
       <c r="I84">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.3895611507651858E-3</v>
       </c>
     </row>
-    <row r="85" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9" ht="42.75">
       <c r="A85" s="1" t="s">
         <v>84</v>
       </c>
@@ -14675,11 +14677,11 @@
         <v>1.36314451735624</v>
       </c>
       <c r="I85">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.6197627601951948E-3</v>
       </c>
     </row>
-    <row r="86" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:9" ht="42.75">
       <c r="A86" s="1" t="s">
         <v>85</v>
       </c>
@@ -14705,11 +14707,11 @@
         <v>1.3621813838522101</v>
       </c>
       <c r="I86">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.1346993579133416E-3</v>
       </c>
     </row>
-    <row r="87" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9" ht="42.75">
       <c r="A87" s="1" t="s">
         <v>86</v>
       </c>
@@ -14735,11 +14737,11 @@
         <v>1.3604310530677299</v>
       </c>
       <c r="I87">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.4511616531233084E-3</v>
       </c>
     </row>
-    <row r="88" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9" ht="42.75">
       <c r="A88" s="1" t="s">
         <v>87</v>
       </c>
@@ -14765,11 +14767,11 @@
         <v>1.3609791880573601</v>
       </c>
       <c r="I88">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.9359041438077277E-3</v>
       </c>
     </row>
-    <row r="89" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9" ht="42.75">
       <c r="A89" s="1" t="s">
         <v>88</v>
       </c>
@@ -14795,11 +14797,11 @@
         <v>1.3613492941684799</v>
       </c>
       <c r="I89">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.855310420222407E-3</v>
       </c>
     </row>
-    <row r="90" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9" ht="42.75">
       <c r="A90" s="1" t="s">
         <v>89</v>
       </c>
@@ -14825,11 +14827,11 @@
         <v>1.3558691857965</v>
       </c>
       <c r="I90">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.3562980491984254E-3</v>
       </c>
     </row>
-    <row r="91" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9" ht="42.75">
       <c r="A91" s="1" t="s">
         <v>90</v>
       </c>
@@ -14855,11 +14857,11 @@
         <v>1.3527725958885599</v>
       </c>
       <c r="I91">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.7894919361514706E-3</v>
       </c>
     </row>
-    <row r="92" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9" ht="42.75">
       <c r="A92" s="1" t="s">
         <v>91</v>
       </c>
@@ -14885,11 +14887,11 @@
         <v>1.35269482603974</v>
       </c>
       <c r="I92">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.7468356623023935E-3</v>
       </c>
     </row>
-    <row r="93" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9" ht="42.75">
       <c r="A93" s="1" t="s">
         <v>92</v>
       </c>
@@ -14915,11 +14917,11 @@
         <v>1.3548054354555199</v>
       </c>
       <c r="I93">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.8721802495066566E-3</v>
       </c>
     </row>
-    <row r="94" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9" ht="42.75">
       <c r="A94" s="1" t="s">
         <v>93</v>
       </c>
@@ -14945,11 +14947,11 @@
         <v>1.3548636727979899</v>
       </c>
       <c r="I94">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.6967420208224219E-3</v>
       </c>
     </row>
-    <row r="95" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9" ht="42.75">
       <c r="A95" s="1" t="s">
         <v>94</v>
       </c>
@@ -14975,11 +14977,11 @@
         <v>1.35107234763887</v>
       </c>
       <c r="I95">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5736165481757534E-3</v>
       </c>
     </row>
-    <row r="96" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:9" ht="42.75">
       <c r="A96" s="1" t="s">
         <v>95</v>
       </c>
@@ -15005,11 +15007,11 @@
         <v>1.3537903697437399</v>
       </c>
       <c r="I96">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.2334809412371663E-3</v>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9" ht="42.75">
       <c r="A97" s="1" t="s">
         <v>96</v>
       </c>
@@ -15035,11 +15037,11 @@
         <v>1.3529420781851</v>
       </c>
       <c r="I97">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.3388927994768237E-3</v>
       </c>
     </row>
-    <row r="98" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9" ht="42.75">
       <c r="A98" s="1" t="s">
         <v>97</v>
       </c>
@@ -15065,11 +15067,11 @@
         <v>1.3517490194786399</v>
       </c>
       <c r="I98">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.7581300531968715E-3</v>
       </c>
     </row>
-    <row r="99" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9" ht="42.75">
       <c r="A99" s="1" t="s">
         <v>98</v>
       </c>
@@ -15095,11 +15097,11 @@
         <v>1.3456728671223801</v>
       </c>
       <c r="I99">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.1611000725158371E-3</v>
       </c>
     </row>
-    <row r="100" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9" ht="42.75">
       <c r="A100" s="1" t="s">
         <v>99</v>
       </c>
@@ -15125,11 +15127,11 @@
         <v>1.35941884756105</v>
       </c>
       <c r="I100">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.2312817866554555E-3</v>
       </c>
     </row>
-    <row r="101" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9" ht="42.75">
       <c r="A101" s="1" t="s">
         <v>100</v>
       </c>
@@ -15155,11 +15157,11 @@
         <v>1.3512711125686201</v>
       </c>
       <c r="I101">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.4166240125878522E-3</v>
       </c>
     </row>
-    <row r="102" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9" ht="42.75">
       <c r="A102" s="1" t="s">
         <v>101</v>
       </c>
@@ -15185,11 +15187,11 @@
         <v>1.34974420815822</v>
       </c>
       <c r="I102">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.0906558551506047E-3</v>
       </c>
     </row>
-    <row r="103" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9" ht="42.75">
       <c r="A103" s="1" t="s">
         <v>102</v>
       </c>
@@ -15215,11 +15217,11 @@
         <v>1.3540146773350299</v>
       </c>
       <c r="I103">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.2474243673122796E-3</v>
       </c>
     </row>
-    <row r="104" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9" ht="42.75">
       <c r="A104" s="1" t="s">
         <v>103</v>
       </c>
@@ -15245,11 +15247,11 @@
         <v>1.35629372876288</v>
       </c>
       <c r="I104">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.8939631737450781E-3</v>
       </c>
     </row>
-    <row r="105" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:9" ht="42.75">
       <c r="A105" s="1" t="s">
         <v>104</v>
       </c>
@@ -15275,11 +15277,11 @@
         <v>1.3520962373352501</v>
       </c>
       <c r="I105">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.15686144924932E-3</v>
       </c>
     </row>
-    <row r="106" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9" ht="42.75">
       <c r="A106" s="1" t="s">
         <v>105</v>
       </c>
@@ -15305,11 +15307,11 @@
         <v>1.3565685046526901</v>
       </c>
       <c r="I106">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1.8658379475729493E-3</v>
       </c>
     </row>
-    <row r="107" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9" ht="42.75">
       <c r="A107" s="1" t="s">
         <v>106</v>
       </c>
@@ -15335,11 +15337,11 @@
         <v>1.34781540878207</v>
       </c>
       <c r="I107">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.7517041952700503E-3</v>
       </c>
     </row>
-    <row r="108" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9" ht="42.75">
       <c r="A108" s="1" t="s">
         <v>107</v>
       </c>
@@ -15365,11 +15367,11 @@
         <v>1.34637174402777</v>
       </c>
       <c r="I108">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.2265784676077606E-3</v>
       </c>
     </row>
-    <row r="109" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9" ht="42.75">
       <c r="A109" s="1" t="s">
         <v>108</v>
       </c>
@@ -15395,11 +15397,11 @@
         <v>1.35204576712438</v>
       </c>
       <c r="I109">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.3148786877302992E-3</v>
       </c>
     </row>
-    <row r="110" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9" ht="42.75">
       <c r="A110" s="1" t="s">
         <v>109</v>
       </c>
@@ -15425,11 +15427,11 @@
         <v>1.3469758396384299</v>
       </c>
       <c r="I110">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.402139728843497E-3</v>
       </c>
     </row>
-    <row r="111" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:9" ht="42.75">
       <c r="A111" s="1" t="s">
         <v>110</v>
       </c>
@@ -15455,11 +15457,11 @@
         <v>1.34878668910799</v>
       </c>
       <c r="I111">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.0343491013099704E-3</v>
       </c>
     </row>
-    <row r="112" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9" ht="42.75">
       <c r="A112" s="1" t="s">
         <v>111</v>
       </c>
@@ -15485,11 +15487,11 @@
         <v>1.34879234924451</v>
       </c>
       <c r="I112">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5179231366855514E-3</v>
       </c>
     </row>
-    <row r="113" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:9" ht="42.75">
       <c r="A113" s="1" t="s">
         <v>112</v>
       </c>
@@ -15515,11 +15517,11 @@
         <v>1.3499162635634301</v>
       </c>
       <c r="I113">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.4921718606836767E-3</v>
       </c>
     </row>
-    <row r="114" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:9" ht="42.75">
       <c r="A114" s="1" t="s">
         <v>113</v>
       </c>
@@ -15545,11 +15547,11 @@
         <v>1.35531174459336</v>
       </c>
       <c r="I114">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.3394411228831935E-3</v>
       </c>
     </row>
-    <row r="115" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:9" ht="42.75">
       <c r="A115" s="1" t="s">
         <v>114</v>
       </c>
@@ -15575,11 +15577,11 @@
         <v>1.3576199254563199</v>
       </c>
       <c r="I115">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.6216795536810975E-3</v>
       </c>
     </row>
-    <row r="116" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:9" ht="42.75">
       <c r="A116" s="1" t="s">
         <v>115</v>
       </c>
@@ -15605,11 +15607,11 @@
         <v>1.35289258891205</v>
       </c>
       <c r="I116">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.5043406083812667E-3</v>
       </c>
     </row>
-    <row r="117" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:9" ht="42.75">
       <c r="A117" s="1" t="s">
         <v>116</v>
       </c>
@@ -15635,11 +15637,11 @@
         <v>1.3509820557475201</v>
       </c>
       <c r="I117">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.6036625944414636E-3</v>
       </c>
     </row>
-    <row r="118" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9" ht="42.75">
       <c r="A118" s="1" t="s">
         <v>117</v>
       </c>
@@ -15665,11 +15667,11 @@
         <v>1.3495913504474399</v>
       </c>
       <c r="I118">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.0306527212468535E-3</v>
       </c>
     </row>
-    <row r="119" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:9" ht="42.75">
       <c r="A119" s="1" t="s">
         <v>118</v>
       </c>
@@ -15695,11 +15697,11 @@
         <v>1.35541891180216</v>
       </c>
       <c r="I119">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.4450384703042839E-3</v>
       </c>
     </row>
-    <row r="120" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:9" ht="42.75">
       <c r="A120" s="1" t="s">
         <v>119</v>
       </c>
@@ -15725,11 +15727,11 @@
         <v>1.35441242806457</v>
       </c>
       <c r="I120">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.6414564178966404E-3</v>
       </c>
     </row>
-    <row r="121" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:9" ht="42.75">
       <c r="A121" s="1" t="s">
         <v>120</v>
       </c>
@@ -15755,11 +15757,11 @@
         <v>1.3541088234018099</v>
       </c>
       <c r="I121">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.430385296613932E-3</v>
       </c>
     </row>
-    <row r="122" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:9" ht="42.75">
       <c r="A122" s="1" t="s">
         <v>121</v>
       </c>
@@ -15785,11 +15787,11 @@
         <v>1.35463803664382</v>
       </c>
       <c r="I122">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.6679430207309971E-3</v>
       </c>
     </row>
-    <row r="123" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:9" ht="42.75">
       <c r="A123" s="1" t="s">
         <v>122</v>
       </c>
@@ -15815,11 +15817,11 @@
         <v>1.3448942376747799</v>
       </c>
       <c r="I123">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.7285821685306528E-3</v>
       </c>
     </row>
-    <row r="124" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:9" ht="42.75">
       <c r="A124" s="1" t="s">
         <v>123</v>
       </c>
@@ -15845,11 +15847,11 @@
         <v>1.3495499097413199</v>
       </c>
       <c r="I124">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.4911660709099862E-3</v>
       </c>
     </row>
-    <row r="125" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:9" ht="42.75">
       <c r="A125" s="1" t="s">
         <v>124</v>
       </c>
@@ -15875,11 +15877,11 @@
         <v>1.3526561390999099</v>
       </c>
       <c r="I125">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.025356833472906E-3</v>
       </c>
     </row>
-    <row r="126" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:9" ht="42.75">
       <c r="A126" s="1" t="s">
         <v>125</v>
       </c>
@@ -15905,11 +15907,11 @@
         <v>1.3489383541184301</v>
       </c>
       <c r="I126">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>3.4281129846071437E-3</v>
       </c>
     </row>
-    <row r="127" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:9" ht="42.75">
       <c r="A127" s="1" t="s">
         <v>126</v>
       </c>
@@ -15935,11 +15937,11 @@
         <v>1.35640708755865</v>
       </c>
       <c r="I127">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.2575246929883918E-3</v>
       </c>
     </row>
-    <row r="128" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:9" ht="42.75">
       <c r="A128" s="1" t="s">
         <v>127</v>
       </c>
@@ -15965,11 +15967,11 @@
         <v>1.3508851090448299</v>
       </c>
       <c r="I128">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.2737765743601787E-3</v>
       </c>
     </row>
-    <row r="129" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:9" ht="42.75">
       <c r="A129" s="1" t="s">
         <v>128</v>
       </c>
@@ -15995,11 +15997,11 @@
         <v>1.35197159858149</v>
       </c>
       <c r="I129">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2.4310795324367987E-3</v>
       </c>
     </row>
-    <row r="130" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:9" ht="42.75">
       <c r="A130" s="1" t="s">
         <v>129</v>
       </c>
@@ -16025,11 +16027,11 @@
         <v>1.3472929616014999</v>
       </c>
       <c r="I130">
-        <f t="shared" ref="I130:I184" si="2">G130/H130</f>
+        <f t="shared" ref="I130:I184" si="3">G130/H130</f>
         <v>2.1679262497918835E-3</v>
       </c>
     </row>
-    <row r="131" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:9" ht="42.75">
       <c r="A131" s="1" t="s">
         <v>0</v>
       </c>
@@ -16055,11 +16057,11 @@
         <v>1.3388372933986199</v>
       </c>
       <c r="I131">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5.3931208293138168E-3</v>
       </c>
     </row>
-    <row r="132" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:9" ht="42.75">
       <c r="A132" s="1" t="s">
         <v>1</v>
       </c>
@@ -16085,11 +16087,11 @@
         <v>1.34164808621162</v>
       </c>
       <c r="I132">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.9969669493333674E-3</v>
       </c>
     </row>
-    <row r="133" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:9" ht="42.75">
       <c r="A133" s="1" t="s">
         <v>2</v>
       </c>
@@ -16115,11 +16117,11 @@
         <v>1.3378072444151301</v>
       </c>
       <c r="I133">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5.0012518152433546E-3</v>
       </c>
     </row>
-    <row r="134" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:9" ht="42.75">
       <c r="A134" s="1" t="s">
         <v>3</v>
       </c>
@@ -16145,11 +16147,11 @@
         <v>1.3389357316571699</v>
       </c>
       <c r="I134">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.7770433366768677E-3</v>
       </c>
     </row>
-    <row r="135" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:9" ht="42.75">
       <c r="A135" s="1" t="s">
         <v>4</v>
       </c>
@@ -16175,11 +16177,11 @@
         <v>1.33910707227475</v>
       </c>
       <c r="I135">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.7905109826317143E-3</v>
       </c>
     </row>
-    <row r="136" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:9" ht="42.75">
       <c r="A136" s="1" t="s">
         <v>5</v>
       </c>
@@ -16205,11 +16207,11 @@
         <v>1.34312554893089</v>
       </c>
       <c r="I136">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.7826951804041231E-3</v>
       </c>
     </row>
-    <row r="137" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:9" ht="42.75">
       <c r="A137" s="1" t="s">
         <v>6</v>
       </c>
@@ -16235,11 +16237,11 @@
         <v>1.34271180018759</v>
       </c>
       <c r="I137">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.2391434815920283E-3</v>
       </c>
     </row>
-    <row r="138" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:9" ht="42.75">
       <c r="A138" s="1" t="s">
         <v>7</v>
       </c>
@@ -16265,11 +16267,11 @@
         <v>1.3442500684432199</v>
       </c>
       <c r="I138">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.0764188211235928E-3</v>
       </c>
     </row>
-    <row r="139" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:9" ht="42.75">
       <c r="A139" s="1" t="s">
         <v>8</v>
       </c>
@@ -16295,11 +16297,11 @@
         <v>1.34526764433837</v>
       </c>
       <c r="I139">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.2869435611514392E-3</v>
       </c>
     </row>
-    <row r="140" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:9" ht="42.75">
       <c r="A140" s="1" t="s">
         <v>9</v>
       </c>
@@ -16325,11 +16327,11 @@
         <v>1.3466219529658701</v>
       </c>
       <c r="I140">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.6517370246778409E-3</v>
       </c>
     </row>
-    <row r="141" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:9" ht="42.75">
       <c r="A141" s="1" t="s">
         <v>10</v>
       </c>
@@ -16355,11 +16357,11 @@
         <v>1.34626876681851</v>
       </c>
       <c r="I141">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.1146858851064646E-3</v>
       </c>
     </row>
-    <row r="142" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:9" ht="42.75">
       <c r="A142" s="1" t="s">
         <v>11</v>
       </c>
@@ -16385,11 +16387,11 @@
         <v>1.34751484466805</v>
       </c>
       <c r="I142">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.7493062915733384E-3</v>
       </c>
     </row>
-    <row r="143" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:9" ht="42.75">
       <c r="A143" s="1" t="s">
         <v>12</v>
       </c>
@@ -16415,11 +16417,11 @@
         <v>1.34620032703981</v>
       </c>
       <c r="I143">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.2163702103224319E-3</v>
       </c>
     </row>
-    <row r="144" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:9" ht="42.75">
       <c r="A144" s="1" t="s">
         <v>13</v>
       </c>
@@ -16445,11 +16447,11 @@
         <v>1.3464130262784499</v>
       </c>
       <c r="I144">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.6619869311992682E-3</v>
       </c>
     </row>
-    <row r="145" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:9" ht="42.75">
       <c r="A145" s="1" t="s">
         <v>14</v>
       </c>
@@ -16475,11 +16477,11 @@
         <v>1.34736977430689</v>
       </c>
       <c r="I145">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4.3975419135405059E-3</v>
       </c>
     </row>
-    <row r="146" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:9" ht="42.75">
       <c r="A146" s="1" t="s">
         <v>15</v>
       </c>
@@ -16505,11 +16507,11 @@
         <v>1.3476102521672</v>
       </c>
       <c r="I146">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.6874396263607977E-3</v>
       </c>
     </row>
-    <row r="147" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:9" ht="42.75">
       <c r="A147" s="1" t="s">
         <v>16</v>
       </c>
@@ -16535,11 +16537,11 @@
         <v>1.34779680141764</v>
       </c>
       <c r="I147">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.4839932128115543E-3</v>
       </c>
     </row>
-    <row r="148" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:9" ht="42.75">
       <c r="A148" s="1" t="s">
         <v>17</v>
       </c>
@@ -16565,11 +16567,11 @@
         <v>1.3481852077832499</v>
       </c>
       <c r="I148">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.9140897538079639E-3</v>
       </c>
     </row>
-    <row r="149" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:9" ht="42.75">
       <c r="A149" s="1" t="s">
         <v>18</v>
       </c>
@@ -16595,11 +16597,11 @@
         <v>1.3483495437906601</v>
       </c>
       <c r="I149">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.1168917514904798E-3</v>
       </c>
     </row>
-    <row r="150" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:9" ht="42.75">
       <c r="A150" s="1" t="s">
         <v>19</v>
       </c>
@@ -16625,11 +16627,11 @@
         <v>1.34753181213934</v>
       </c>
       <c r="I150">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.9679149715213333E-3</v>
       </c>
     </row>
-    <row r="151" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:9" ht="42.75">
       <c r="A151" s="1" t="s">
         <v>20</v>
       </c>
@@ -16655,11 +16657,11 @@
         <v>1.3481108648590601</v>
       </c>
       <c r="I151">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.7851461918386423E-3</v>
       </c>
     </row>
-    <row r="152" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:9" ht="42.75">
       <c r="A152" s="1" t="s">
         <v>21</v>
       </c>
@@ -16685,11 +16687,11 @@
         <v>1.34690899692844</v>
       </c>
       <c r="I152">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.6576508356238051E-3</v>
       </c>
     </row>
-    <row r="153" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:9" ht="42.75">
       <c r="A153" s="1" t="s">
         <v>22</v>
       </c>
@@ -16715,11 +16717,11 @@
         <v>1.3460335494212099</v>
       </c>
       <c r="I153">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3.5271693280876622E-3</v>
       </c>
     </row>
-    <row r="154" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:9" ht="42.75">
       <c r="A154" s="1" t="s">
         <v>130</v>
       </c>
@@ -16745,11 +16747,11 @@
         <v>1.34270192424532</v>
       </c>
       <c r="I154">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.668437060479016E-3</v>
       </c>
     </row>
-    <row r="155" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:9" ht="42.75">
       <c r="A155" s="1" t="s">
         <v>131</v>
       </c>
@@ -16775,11 +16777,11 @@
         <v>1.34162370844164</v>
       </c>
       <c r="I155">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.6953994989720423E-3</v>
       </c>
     </row>
-    <row r="156" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:9" ht="42.75">
       <c r="A156" s="1" t="s">
         <v>132</v>
       </c>
@@ -16805,11 +16807,11 @@
         <v>1.3387352184102099</v>
       </c>
       <c r="I156">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.2553218464812694E-3</v>
       </c>
     </row>
-    <row r="157" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:9" ht="42.75">
       <c r="A157" s="1" t="s">
         <v>133</v>
       </c>
@@ -16835,11 +16837,11 @@
         <v>1.3440198413078099</v>
       </c>
       <c r="I157">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7888972677859074E-3</v>
       </c>
     </row>
-    <row r="158" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:9" ht="42.75">
       <c r="A158" s="1" t="s">
         <v>134</v>
       </c>
@@ -16865,11 +16867,11 @@
         <v>1.3424657372509901</v>
       </c>
       <c r="I158">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2.2045773550842833E-3</v>
       </c>
     </row>
-    <row r="159" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:9" ht="42.75">
       <c r="A159" s="1" t="s">
         <v>135</v>
       </c>
@@ -16895,11 +16897,11 @@
         <v>1.3416755441102099</v>
       </c>
       <c r="I159">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1389074448513172E-3</v>
       </c>
     </row>
-    <row r="160" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:9" ht="42.75">
       <c r="A160" s="1" t="s">
         <v>136</v>
       </c>
@@ -16925,11 +16927,11 @@
         <v>1.3413881668657299</v>
       </c>
       <c r="I160">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7883088819000343E-3</v>
       </c>
     </row>
-    <row r="161" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:9" ht="42.75">
       <c r="A161" s="1" t="s">
         <v>137</v>
       </c>
@@ -16955,11 +16957,11 @@
         <v>1.3416244306357401</v>
       </c>
       <c r="I161">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1188471714718581E-3</v>
       </c>
     </row>
-    <row r="162" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:9" ht="42.75">
       <c r="A162" s="1" t="s">
         <v>138</v>
       </c>
@@ -16985,11 +16987,11 @@
         <v>1.34519999115509</v>
       </c>
       <c r="I162">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7757870071851815E-3</v>
       </c>
     </row>
-    <row r="163" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:9" ht="42.75">
       <c r="A163" s="1" t="s">
         <v>139</v>
       </c>
@@ -17015,11 +17017,11 @@
         <v>1.34569446103736</v>
       </c>
       <c r="I163">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.2819393639065865E-3</v>
       </c>
     </row>
-    <row r="164" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:9" ht="42.75">
       <c r="A164" s="1" t="s">
         <v>140</v>
       </c>
@@ -17045,11 +17047,11 @@
         <v>1.34790011041296</v>
       </c>
       <c r="I164">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.6124313880359728E-3</v>
       </c>
     </row>
-    <row r="165" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:9" ht="42.75">
       <c r="A165" s="1" t="s">
         <v>141</v>
       </c>
@@ -17075,11 +17077,11 @@
         <v>1.3472363205996001</v>
       </c>
       <c r="I165">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7580075162695944E-3</v>
       </c>
     </row>
-    <row r="166" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:9" ht="42.75">
       <c r="A166" s="1" t="s">
         <v>142</v>
       </c>
@@ -17105,11 +17107,11 @@
         <v>1.3487252797182501</v>
       </c>
       <c r="I166">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.1565776709209646E-3</v>
       </c>
     </row>
-    <row r="167" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:9" ht="42.75">
       <c r="A167" s="1" t="s">
         <v>143</v>
       </c>
@@ -17135,11 +17137,11 @@
         <v>1.3503816157127799</v>
       </c>
       <c r="I167">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3928163991348242E-3</v>
       </c>
     </row>
-    <row r="168" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:9" ht="42.75">
       <c r="A168" s="1" t="s">
         <v>144</v>
       </c>
@@ -17165,11 +17167,11 @@
         <v>1.3476697714486101</v>
       </c>
       <c r="I168">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.5449844433552368E-3</v>
       </c>
     </row>
-    <row r="169" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:9" ht="42.75">
       <c r="A169" s="1" t="s">
         <v>145</v>
       </c>
@@ -17195,11 +17197,11 @@
         <v>1.3439767091925801</v>
       </c>
       <c r="I169">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3704743971168878E-3</v>
       </c>
     </row>
-    <row r="170" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:9" ht="42.75">
       <c r="A170" s="1" t="s">
         <v>146</v>
       </c>
@@ -17225,11 +17227,11 @@
         <v>1.3465038614372</v>
       </c>
       <c r="I170">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.611793361861466E-3</v>
       </c>
     </row>
-    <row r="171" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:9" ht="42.75">
       <c r="A171" s="1" t="s">
         <v>147</v>
       </c>
@@ -17255,11 +17257,11 @@
         <v>1.3472171016888299</v>
       </c>
       <c r="I171">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9.2228013018254122E-4</v>
       </c>
     </row>
-    <row r="172" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:9" ht="42.75">
       <c r="A172" s="1" t="s">
         <v>148</v>
       </c>
@@ -17285,11 +17287,11 @@
         <v>1.3498146773278901</v>
       </c>
       <c r="I172">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3537631648619082E-3</v>
       </c>
     </row>
-    <row r="173" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:9" ht="42.75">
       <c r="A173" s="1" t="s">
         <v>149</v>
       </c>
@@ -17315,11 +17317,11 @@
         <v>1.3483720352917301</v>
       </c>
       <c r="I173">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7678370759310125E-3</v>
       </c>
     </row>
-    <row r="174" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:9" ht="42.75">
       <c r="A174" s="1" t="s">
         <v>150</v>
       </c>
@@ -17345,11 +17347,11 @@
         <v>1.3514102514083099</v>
       </c>
       <c r="I174">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3027365052746887E-3</v>
       </c>
     </row>
-    <row r="175" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:9" ht="42.75">
       <c r="A175" s="1" t="s">
         <v>151</v>
       </c>
@@ -17375,11 +17377,11 @@
         <v>1.35097859448045</v>
       </c>
       <c r="I175">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3869629509612672E-3</v>
       </c>
     </row>
-    <row r="176" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:9" ht="42.75">
       <c r="A176" s="1" t="s">
         <v>152</v>
       </c>
@@ -17405,11 +17407,11 @@
         <v>1.35124692357133</v>
       </c>
       <c r="I176">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.0256882048060535E-3</v>
       </c>
     </row>
-    <row r="177" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:19" ht="42.75">
       <c r="A177" s="1" t="s">
         <v>153</v>
       </c>
@@ -17435,11 +17437,11 @@
         <v>1.35318508485804</v>
       </c>
       <c r="I177">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.611027331554509E-3</v>
       </c>
     </row>
-    <row r="178" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:19" ht="42.75">
       <c r="A178" s="1" t="s">
         <v>154</v>
       </c>
@@ -17465,11 +17467,11 @@
         <v>1.3536617533647199</v>
       </c>
       <c r="I178">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.669911408246747E-3</v>
       </c>
     </row>
-    <row r="179" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:19" ht="42.75">
       <c r="A179" s="1" t="s">
         <v>155</v>
       </c>
@@ -17495,11 +17497,11 @@
         <v>1.3494901062514599</v>
       </c>
       <c r="I179">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.8705643171407795E-3</v>
       </c>
     </row>
-    <row r="180" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:19" ht="42.75">
       <c r="A180" s="1" t="s">
         <v>156</v>
       </c>
@@ -17525,11 +17527,11 @@
         <v>1.34876818148872</v>
       </c>
       <c r="I180">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.7647609594323951E-3</v>
       </c>
     </row>
-    <row r="181" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:19" ht="42.75">
       <c r="A181" s="1" t="s">
         <v>157</v>
       </c>
@@ -17555,11 +17557,11 @@
         <v>1.3502568614847701</v>
       </c>
       <c r="I181">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.6705235794169241E-3</v>
       </c>
     </row>
-    <row r="182" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:19" ht="42.75">
       <c r="A182" s="1" t="s">
         <v>158</v>
       </c>
@@ -17585,11 +17587,11 @@
         <v>1.3511680362248699</v>
       </c>
       <c r="I182">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.6940174300061864E-3</v>
       </c>
     </row>
-    <row r="183" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:19" ht="42.75">
       <c r="A183" s="1" t="s">
         <v>159</v>
       </c>
@@ -17615,11 +17617,11 @@
         <v>1.3509224556673101</v>
       </c>
       <c r="I183">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.3633786828254873E-3</v>
       </c>
     </row>
-    <row r="184" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:19" ht="42.75">
       <c r="A184" s="1" t="s">
         <v>160</v>
       </c>
@@ -17645,11 +17647,11 @@
         <v>1.3447068396988</v>
       </c>
       <c r="I184">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1.975036306037702E-3</v>
       </c>
     </row>
-    <row r="185" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:19" ht="42.75">
       <c r="K185" s="1" t="s">
         <v>161</v>
       </c>
@@ -17675,11 +17677,11 @@
         <v>1.3688711685145001</v>
       </c>
       <c r="S185">
-        <f>Q185/R185</f>
+        <f t="shared" ref="S185:S209" si="4">Q185/R185</f>
         <v>4.7498021587517401E-3</v>
       </c>
     </row>
-    <row r="186" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:19" ht="42.75">
       <c r="K186" s="1" t="s">
         <v>162</v>
       </c>
@@ -17705,11 +17707,11 @@
         <v>1.3702983184380499</v>
       </c>
       <c r="S186">
-        <f>Q186/R186</f>
+        <f t="shared" si="4"/>
         <v>4.582077330036116E-3</v>
       </c>
     </row>
-    <row r="187" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:19" ht="42.75">
       <c r="K187" s="1" t="s">
         <v>163</v>
       </c>
@@ -17735,11 +17737,11 @@
         <v>1.3695888476757001</v>
       </c>
       <c r="S187">
-        <f>Q187/R187</f>
+        <f t="shared" si="4"/>
         <v>5.4048359998903461E-3</v>
       </c>
     </row>
-    <row r="188" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:19" ht="42.75">
       <c r="K188" s="1" t="s">
         <v>164</v>
       </c>
@@ -17765,11 +17767,11 @@
         <v>1.3632148140396101</v>
       </c>
       <c r="S188">
-        <f>Q188/R188</f>
+        <f t="shared" si="4"/>
         <v>5.0546032246706401E-3</v>
       </c>
     </row>
-    <row r="189" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:19" ht="42.75">
       <c r="K189" s="1" t="s">
         <v>165</v>
       </c>
@@ -17795,11 +17797,11 @@
         <v>1.3638903693308999</v>
       </c>
       <c r="S189">
-        <f>Q189/R189</f>
+        <f t="shared" si="4"/>
         <v>4.6950553057131137E-3</v>
       </c>
     </row>
-    <row r="190" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:19" ht="42.75">
       <c r="K190" s="1" t="s">
         <v>166</v>
       </c>
@@ -17825,11 +17827,11 @@
         <v>1.36364377647032</v>
       </c>
       <c r="S190">
-        <f>Q190/R190</f>
+        <f t="shared" si="4"/>
         <v>4.5501515897943077E-3</v>
       </c>
     </row>
-    <row r="191" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:19" ht="42.75">
       <c r="K191" s="1" t="s">
         <v>167</v>
       </c>
@@ -17855,11 +17857,11 @@
         <v>1.3631256441701001</v>
       </c>
       <c r="S191">
-        <f>Q191/R191</f>
+        <f t="shared" si="4"/>
         <v>4.440617995568742E-3</v>
       </c>
     </row>
-    <row r="192" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:19" ht="42.75">
       <c r="K192" s="1" t="s">
         <v>168</v>
       </c>
@@ -17885,11 +17887,11 @@
         <v>1.3639194096987699</v>
       </c>
       <c r="S192">
-        <f>Q192/R192</f>
+        <f t="shared" si="4"/>
         <v>4.6493209293703838E-3</v>
       </c>
     </row>
-    <row r="193" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="193" spans="11:19" ht="42.75">
       <c r="K193" s="1" t="s">
         <v>169</v>
       </c>
@@ -17915,11 +17917,11 @@
         <v>1.3625696954355599</v>
       </c>
       <c r="S193">
-        <f>Q193/R193</f>
+        <f t="shared" si="4"/>
         <v>4.7983404105203693E-3</v>
       </c>
     </row>
-    <row r="194" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="194" spans="11:19" ht="42.75">
       <c r="K194" s="1" t="s">
         <v>170</v>
       </c>
@@ -17945,11 +17947,11 @@
         <v>1.36401667395241</v>
       </c>
       <c r="S194">
-        <f>Q194/R194</f>
+        <f t="shared" si="4"/>
         <v>4.4651418520494542E-3</v>
       </c>
     </row>
-    <row r="195" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="195" spans="11:19" ht="42.75">
       <c r="K195" s="1" t="s">
         <v>171</v>
       </c>
@@ -17975,11 +17977,11 @@
         <v>1.3671347323290299</v>
       </c>
       <c r="S195">
-        <f>Q195/R195</f>
+        <f t="shared" si="4"/>
         <v>5.2314593585967746E-3</v>
       </c>
     </row>
-    <row r="196" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="196" spans="11:19" ht="42.75">
       <c r="K196" s="1" t="s">
         <v>172</v>
       </c>
@@ -18005,11 +18007,11 @@
         <v>1.36692877179062</v>
       </c>
       <c r="S196">
-        <f>Q196/R196</f>
+        <f t="shared" si="4"/>
         <v>4.4725632152429334E-3</v>
       </c>
     </row>
-    <row r="197" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="197" spans="11:19" ht="42.75">
       <c r="K197" s="1" t="s">
         <v>173</v>
       </c>
@@ -18035,11 +18037,11 @@
         <v>1.3663664972381999</v>
       </c>
       <c r="S197">
-        <f>Q197/R197</f>
+        <f t="shared" si="4"/>
         <v>4.2732093372212726E-3</v>
       </c>
     </row>
-    <row r="198" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="198" spans="11:19" ht="42.75">
       <c r="K198" s="1" t="s">
         <v>174</v>
       </c>
@@ -18065,11 +18067,11 @@
         <v>1.3705832023220399</v>
       </c>
       <c r="S198">
-        <f>Q198/R198</f>
+        <f t="shared" si="4"/>
         <v>4.614112376785026E-3</v>
       </c>
     </row>
-    <row r="199" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="199" spans="11:19" ht="42.75">
       <c r="K199" s="1" t="s">
         <v>175</v>
       </c>
@@ -18095,11 +18097,11 @@
         <v>1.3708604781129801</v>
       </c>
       <c r="S199">
-        <f>Q199/R199</f>
+        <f t="shared" si="4"/>
         <v>5.2515909271172558E-3</v>
       </c>
     </row>
-    <row r="200" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="200" spans="11:19" ht="42.75">
       <c r="K200" s="1" t="s">
         <v>176</v>
       </c>
@@ -18125,11 +18127,11 @@
         <v>1.3699218632639401</v>
       </c>
       <c r="S200">
-        <f>Q200/R200</f>
+        <f t="shared" si="4"/>
         <v>5.1891013989471954E-3</v>
       </c>
     </row>
-    <row r="201" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="201" spans="11:19" ht="42.75">
       <c r="K201" s="1" t="s">
         <v>177</v>
       </c>
@@ -18155,11 +18157,11 @@
         <v>1.36998951006876</v>
       </c>
       <c r="S201">
-        <f>Q201/R201</f>
+        <f t="shared" si="4"/>
         <v>5.0166174167543135E-3</v>
       </c>
     </row>
-    <row r="202" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="202" spans="11:19" ht="42.75">
       <c r="K202" s="1" t="s">
         <v>178</v>
       </c>
@@ -18185,11 +18187,11 @@
         <v>1.36956109707921</v>
       </c>
       <c r="S202">
-        <f>Q202/R202</f>
+        <f t="shared" si="4"/>
         <v>5.0675752156878751E-3</v>
       </c>
     </row>
-    <row r="203" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="203" spans="11:19" ht="42.75">
       <c r="K203" s="1" t="s">
         <v>179</v>
       </c>
@@ -18215,11 +18217,11 @@
         <v>1.3679138697989199</v>
       </c>
       <c r="S203">
-        <f>Q203/R203</f>
+        <f t="shared" si="4"/>
         <v>4.5123935532537752E-3</v>
       </c>
     </row>
-    <row r="204" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="204" spans="11:19" ht="42.75">
       <c r="K204" s="1" t="s">
         <v>180</v>
       </c>
@@ -18245,11 +18247,11 @@
         <v>1.3709646451391</v>
       </c>
       <c r="S204">
-        <f>Q204/R204</f>
+        <f t="shared" si="4"/>
         <v>4.8810945370999555E-3</v>
       </c>
     </row>
-    <row r="205" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="205" spans="11:19" ht="42.75">
       <c r="K205" s="1" t="s">
         <v>181</v>
       </c>
@@ -18275,11 +18277,11 @@
         <v>1.36951320598659</v>
       </c>
       <c r="S205">
-        <f>Q205/R205</f>
+        <f t="shared" si="4"/>
         <v>5.3430376625483887E-3</v>
       </c>
     </row>
-    <row r="206" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="206" spans="11:19" ht="42.75">
       <c r="K206" s="1" t="s">
         <v>182</v>
       </c>
@@ -18305,11 +18307,11 @@
         <v>1.37044480265897</v>
       </c>
       <c r="S206">
-        <f>Q206/R206</f>
+        <f t="shared" si="4"/>
         <v>5.0246056566637448E-3</v>
       </c>
     </row>
-    <row r="207" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="207" spans="11:19" ht="42.75">
       <c r="K207" s="1" t="s">
         <v>183</v>
       </c>
@@ -18335,11 +18337,11 @@
         <v>1.3711517444556001</v>
       </c>
       <c r="S207">
-        <f>Q207/R207</f>
+        <f t="shared" si="4"/>
         <v>4.9890546515495128E-3</v>
       </c>
     </row>
-    <row r="208" spans="11:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="208" spans="11:19" ht="42.75">
       <c r="K208" s="1" t="s">
         <v>184</v>
       </c>
@@ -18365,11 +18367,11 @@
         <v>1.36953950454926</v>
       </c>
       <c r="S208">
-        <f>Q208/R208</f>
+        <f t="shared" si="4"/>
         <v>5.0159924603581105E-3</v>
       </c>
     </row>
-    <row r="209" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:19" ht="42.75">
       <c r="K209" s="1" t="s">
         <v>185</v>
       </c>
@@ -18395,11 +18397,11 @@
         <v>1.3665184240166199</v>
       </c>
       <c r="S209">
-        <f>Q209/R209</f>
+        <f t="shared" si="4"/>
         <v>4.7919428036830025E-3</v>
       </c>
     </row>
-    <row r="210" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:19" ht="42.75">
       <c r="A210" s="1" t="s">
         <v>186</v>
       </c>
@@ -18425,11 +18427,11 @@
         <v>1.3436143758649299</v>
       </c>
       <c r="I210">
-        <f t="shared" ref="I210:I257" si="3">G210/H210</f>
+        <f t="shared" ref="I210:I257" si="5">G210/H210</f>
         <v>7.7533610308483673E-4</v>
       </c>
     </row>
-    <row r="211" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:19" ht="42.75">
       <c r="A211" s="1" t="s">
         <v>187</v>
       </c>
@@ -18455,11 +18457,11 @@
         <v>1.3420054527155301</v>
       </c>
       <c r="I211">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.1489061309278147E-3</v>
       </c>
     </row>
-    <row r="212" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:19" ht="42.75">
       <c r="A212" s="1" t="s">
         <v>188</v>
       </c>
@@ -18485,11 +18487,11 @@
         <v>1.35078765083904</v>
       </c>
       <c r="I212">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>7.6156331327219935E-4</v>
       </c>
     </row>
-    <row r="213" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:19" ht="42.75">
       <c r="A213" s="1" t="s">
         <v>189</v>
       </c>
@@ -18515,11 +18517,11 @@
         <v>1.34844793264089</v>
       </c>
       <c r="I213">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>7.6835191432661932E-4</v>
       </c>
     </row>
-    <row r="214" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:19" ht="42.75">
       <c r="A214" s="1" t="s">
         <v>190</v>
       </c>
@@ -18545,11 +18547,11 @@
         <v>1.3494952442163799</v>
       </c>
       <c r="I214">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>8.0116063073005909E-4</v>
       </c>
     </row>
-    <row r="215" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:19" ht="42.75">
       <c r="A215" s="1" t="s">
         <v>191</v>
       </c>
@@ -18575,11 +18577,11 @@
         <v>1.34302893816314</v>
       </c>
       <c r="I215">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.2044030403225786E-3</v>
       </c>
     </row>
-    <row r="216" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:19" ht="42.75">
       <c r="A216" s="1" t="s">
         <v>192</v>
       </c>
@@ -18605,11 +18607,11 @@
         <v>1.3413715402622599</v>
       </c>
       <c r="I216">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.3665050897021946E-4</v>
       </c>
     </row>
-    <row r="217" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:19" ht="42.75">
       <c r="A217" s="1" t="s">
         <v>193</v>
       </c>
@@ -18635,11 +18637,11 @@
         <v>1.34690075729866</v>
       </c>
       <c r="I217">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.3316703366491414E-3</v>
       </c>
     </row>
-    <row r="218" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:19" ht="42.75">
       <c r="A218" s="1" t="s">
         <v>194</v>
       </c>
@@ -18665,11 +18667,11 @@
         <v>1.3399150016652901</v>
       </c>
       <c r="I218">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.2225644965498671E-4</v>
       </c>
     </row>
-    <row r="219" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:19" ht="42.75">
       <c r="A219" s="1" t="s">
         <v>195</v>
       </c>
@@ -18695,11 +18697,11 @@
         <v>1.3450766964337799</v>
       </c>
       <c r="I219">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.532689486873119E-4</v>
       </c>
     </row>
-    <row r="220" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:19" ht="42.75">
       <c r="A220" s="1" t="s">
         <v>196</v>
       </c>
@@ -18725,11 +18727,11 @@
         <v>1.3461650995699199</v>
       </c>
       <c r="I220">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.7910422616618434E-4</v>
       </c>
     </row>
-    <row r="221" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:19" ht="42.75">
       <c r="A221" s="1" t="s">
         <v>197</v>
       </c>
@@ -18755,11 +18757,11 @@
         <v>1.34267977050327</v>
       </c>
       <c r="I221">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>6.1181089861039829E-4</v>
       </c>
     </row>
-    <row r="222" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:19" ht="42.75">
       <c r="A222" s="1" t="s">
         <v>198</v>
       </c>
@@ -18785,11 +18787,11 @@
         <v>1.3434234724585601</v>
       </c>
       <c r="I222">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.0002642776588755E-3</v>
       </c>
     </row>
-    <row r="223" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:19" ht="42.75">
       <c r="A223" s="1" t="s">
         <v>199</v>
       </c>
@@ -18815,11 +18817,11 @@
         <v>1.3469035667615099</v>
       </c>
       <c r="I223">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>4.4725880372957304E-4</v>
       </c>
     </row>
-    <row r="224" spans="1:19" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:19" ht="42.75">
       <c r="A224" s="1" t="s">
         <v>200</v>
       </c>
@@ -18845,11 +18847,11 @@
         <v>1.34733691880411</v>
       </c>
       <c r="I224">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.4346139136026204E-4</v>
       </c>
     </row>
-    <row r="225" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:9" ht="42.75">
       <c r="A225" s="1" t="s">
         <v>201</v>
       </c>
@@ -18875,11 +18877,11 @@
         <v>1.3449071899032401</v>
       </c>
       <c r="I225">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>5.9918547978657258E-4</v>
       </c>
     </row>
-    <row r="226" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:9" ht="42.75">
       <c r="A226" s="1" t="s">
         <v>202</v>
       </c>
@@ -18905,11 +18907,11 @@
         <v>1.3457441226723601</v>
       </c>
       <c r="I226">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.1400435732591074E-3</v>
       </c>
     </row>
-    <row r="227" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:9" ht="42.75">
       <c r="A227" s="1" t="s">
         <v>203</v>
       </c>
@@ -18935,11 +18937,11 @@
         <v>1.3385254683524901</v>
       </c>
       <c r="I227">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>7.8956768813062672E-4</v>
       </c>
     </row>
-    <row r="228" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:9" ht="42.75">
       <c r="A228" s="1" t="s">
         <v>204</v>
       </c>
@@ -18965,11 +18967,11 @@
         <v>1.3452250952112299</v>
       </c>
       <c r="I228">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>4.2144654949038913E-4</v>
       </c>
     </row>
-    <row r="229" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:9" ht="42.75">
       <c r="A229" s="1" t="s">
         <v>205</v>
       </c>
@@ -18995,11 +18997,11 @@
         <v>1.3405022698277</v>
       </c>
       <c r="I229">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.7883439379642017E-4</v>
       </c>
     </row>
-    <row r="230" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:9" ht="42.75">
       <c r="A230" s="1" t="s">
         <v>206</v>
       </c>
@@ -19025,11 +19027,11 @@
         <v>1.3402841356305399</v>
       </c>
       <c r="I230">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>4.0303466408772386E-4</v>
       </c>
     </row>
-    <row r="231" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:9" ht="42.75">
       <c r="A231" s="1" t="s">
         <v>207</v>
       </c>
@@ -19055,11 +19057,11 @@
         <v>1.34474083880747</v>
       </c>
       <c r="I231">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.4120660139062416E-3</v>
       </c>
     </row>
-    <row r="232" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:9" ht="42.75">
       <c r="A232" s="1" t="s">
         <v>208</v>
       </c>
@@ -19085,11 +19087,11 @@
         <v>1.3439324264850201</v>
       </c>
       <c r="I232">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>5.1376285563701596E-4</v>
       </c>
     </row>
-    <row r="233" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:9" ht="42.75">
       <c r="A233" s="1" t="s">
         <v>209</v>
       </c>
@@ -19115,11 +19117,11 @@
         <v>1.3419865588525199</v>
       </c>
       <c r="I233">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.6124462275440745E-3</v>
       </c>
     </row>
-    <row r="234" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:9" ht="42.75">
       <c r="A234" s="1" t="s">
         <v>210</v>
       </c>
@@ -19145,11 +19147,11 @@
         <v>1.3404397486937301</v>
       </c>
       <c r="I234">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>8.5049659310509722E-4</v>
       </c>
     </row>
-    <row r="235" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:9" ht="42.75">
       <c r="A235" s="1" t="s">
         <v>211</v>
       </c>
@@ -19175,11 +19177,11 @@
         <v>1.3401055446138099</v>
       </c>
       <c r="I235">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>8.2720267827902135E-4</v>
       </c>
     </row>
-    <row r="236" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:9" ht="42.75">
       <c r="A236" s="1" t="s">
         <v>212</v>
       </c>
@@ -19205,11 +19207,11 @@
         <v>1.3476608841164801</v>
       </c>
       <c r="I236">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>4.2445922503189977E-4</v>
       </c>
     </row>
-    <row r="237" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:9" ht="42.75">
       <c r="A237" s="1" t="s">
         <v>213</v>
       </c>
@@ -19235,11 +19237,11 @@
         <v>1.3423655180223699</v>
       </c>
       <c r="I237">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>8.6847651569724117E-4</v>
       </c>
     </row>
-    <row r="238" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:9" ht="42.75">
       <c r="A238" s="1" t="s">
         <v>214</v>
       </c>
@@ -19265,11 +19267,11 @@
         <v>1.3428425064823599</v>
       </c>
       <c r="I238">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.6226775287664342E-3</v>
       </c>
     </row>
-    <row r="239" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:9" ht="42.75">
       <c r="A239" s="1" t="s">
         <v>215</v>
       </c>
@@ -19295,11 +19297,11 @@
         <v>1.34359747244184</v>
       </c>
       <c r="I239">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.7549064832154747E-3</v>
       </c>
     </row>
-    <row r="240" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:9" ht="42.75">
       <c r="A240" s="1" t="s">
         <v>216</v>
       </c>
@@ -19325,11 +19327,11 @@
         <v>1.3444634587184301</v>
       </c>
       <c r="I240">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>5.86034877748742E-4</v>
       </c>
     </row>
-    <row r="241" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:9" ht="42.75">
       <c r="A241" s="1" t="s">
         <v>217</v>
       </c>
@@ -19355,11 +19357,11 @@
         <v>1.3449716925441</v>
       </c>
       <c r="I241">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.3881397261864923E-3</v>
       </c>
     </row>
-    <row r="242" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:9" ht="42.75">
       <c r="A242" s="1" t="s">
         <v>218</v>
       </c>
@@ -19385,11 +19387,11 @@
         <v>1.3455862766211699</v>
       </c>
       <c r="I242">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.2475030881067182E-3</v>
       </c>
     </row>
-    <row r="243" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:9" ht="42.75">
       <c r="A243" s="1" t="s">
         <v>219</v>
       </c>
@@ -19415,11 +19417,11 @@
         <v>1.3480306247740299</v>
       </c>
       <c r="I243">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.8450319095371607E-3</v>
       </c>
     </row>
-    <row r="244" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:9" ht="42.75">
       <c r="A244" s="1" t="s">
         <v>220</v>
       </c>
@@ -19445,11 +19447,11 @@
         <v>1.34567111747496</v>
       </c>
       <c r="I244">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>1.208935527723966E-3</v>
       </c>
     </row>
-    <row r="245" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:9" ht="42.75">
       <c r="A245" s="1" t="s">
         <v>221</v>
       </c>
@@ -19475,11 +19477,11 @@
         <v>1.35347045638191</v>
       </c>
       <c r="I245">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.9286729581604553E-3</v>
       </c>
     </row>
-    <row r="246" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:9" ht="42.75">
       <c r="A246" s="1" t="s">
         <v>222</v>
       </c>
@@ -19505,11 +19507,11 @@
         <v>1.35359798487156</v>
       </c>
       <c r="I246">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.8743249147507618E-3</v>
       </c>
     </row>
-    <row r="247" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:9" ht="42.75">
       <c r="A247" s="1" t="s">
         <v>223</v>
       </c>
@@ -19535,11 +19537,11 @@
         <v>1.3550505312226899</v>
       </c>
       <c r="I247">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.1306116817912634E-3</v>
       </c>
     </row>
-    <row r="248" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:9" ht="42.75">
       <c r="A248" s="1" t="s">
         <v>224</v>
       </c>
@@ -19565,11 +19567,11 @@
         <v>1.35428020739886</v>
       </c>
       <c r="I248">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.5566215539300175E-3</v>
       </c>
     </row>
-    <row r="249" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:9" ht="42.75">
       <c r="A249" s="1" t="s">
         <v>225</v>
       </c>
@@ -19595,11 +19597,11 @@
         <v>1.3657120765916599</v>
       </c>
       <c r="I249">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.0354019040875597E-3</v>
       </c>
     </row>
-    <row r="250" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:9" ht="42.75">
       <c r="A250" s="1" t="s">
         <v>226</v>
       </c>
@@ -19625,11 +19627,11 @@
         <v>1.3643824284422399</v>
       </c>
       <c r="I250">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>2.6051302764988687E-3</v>
       </c>
     </row>
-    <row r="251" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:9" ht="42.75">
       <c r="A251" s="1" t="s">
         <v>227</v>
       </c>
@@ -19655,11 +19657,11 @@
         <v>1.3600093982777799</v>
       </c>
       <c r="I251">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.0113553630124737E-3</v>
       </c>
     </row>
-    <row r="252" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:9" ht="42.75">
       <c r="A252" s="1" t="s">
         <v>228</v>
       </c>
@@ -19685,11 +19687,11 @@
         <v>1.35970172222735</v>
       </c>
       <c r="I252">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.3081967638200959E-3</v>
       </c>
     </row>
-    <row r="253" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:9" ht="42.75">
       <c r="A253" s="1" t="s">
         <v>229</v>
       </c>
@@ -19715,11 +19717,11 @@
         <v>1.34950592576274</v>
       </c>
       <c r="I253">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.721521603935238E-3</v>
       </c>
     </row>
-    <row r="254" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:9" ht="42.75">
       <c r="A254" s="1" t="s">
         <v>230</v>
       </c>
@@ -19745,11 +19747,11 @@
         <v>1.3516289575709299</v>
       </c>
       <c r="I254">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.0281179828710691E-3</v>
       </c>
     </row>
-    <row r="255" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:9" ht="42.75">
       <c r="A255" s="1" t="s">
         <v>231</v>
       </c>
@@ -19775,11 +19777,11 @@
         <v>1.35231733901114</v>
       </c>
       <c r="I255">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.6895804749107249E-3</v>
       </c>
     </row>
-    <row r="256" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:9" ht="42.75">
       <c r="A256" s="1" t="s">
         <v>232</v>
       </c>
@@ -19805,11 +19807,11 @@
         <v>1.3524119591633099</v>
       </c>
       <c r="I256">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.0180715939024977E-3</v>
       </c>
     </row>
-    <row r="257" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:9" ht="42.75">
       <c r="A257" s="1" t="s">
         <v>233</v>
       </c>
@@ -19835,11 +19837,11 @@
         <v>1.3548269662139201</v>
       </c>
       <c r="I257">
-        <f t="shared" si="3"/>
+        <f t="shared" si="5"/>
         <v>3.2502064427327578E-3</v>
       </c>
     </row>
-    <row r="258" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:9" ht="42.75">
       <c r="A258" s="1" t="s">
         <v>234</v>
       </c>
@@ -19865,11 +19867,11 @@
         <v>1.35292883897614</v>
       </c>
       <c r="I258">
-        <f t="shared" ref="I258:I308" si="4">G258/H258</f>
+        <f t="shared" ref="I258:I308" si="6">G258/H258</f>
         <v>3.2430711219260879E-3</v>
       </c>
     </row>
-    <row r="259" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:9" ht="42.75">
       <c r="A259" s="1" t="s">
         <v>235</v>
       </c>
@@ -19895,11 +19897,11 @@
         <v>1.3548391979296099</v>
       </c>
       <c r="I259">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.9064704674973958E-3</v>
       </c>
     </row>
-    <row r="260" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:9" ht="42.75">
       <c r="A260" s="1" t="s">
         <v>236</v>
       </c>
@@ -19925,11 +19927,11 @@
         <v>1.3551153167332</v>
       </c>
       <c r="I260">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.1951896098057291E-3</v>
       </c>
     </row>
-    <row r="261" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:9" ht="42.75">
       <c r="A261" s="1" t="s">
         <v>237</v>
       </c>
@@ -19955,11 +19957,11 @@
         <v>1.3585310976191101</v>
       </c>
       <c r="I261">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.4715549619159843E-3</v>
       </c>
     </row>
-    <row r="262" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:9" ht="42.75">
       <c r="A262" s="1" t="s">
         <v>238</v>
       </c>
@@ -19985,11 +19987,11 @@
         <v>1.35947659720951</v>
       </c>
       <c r="I262">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.9272945631826077E-3</v>
       </c>
     </row>
-    <row r="263" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:9" ht="42.75">
       <c r="A263" s="1" t="s">
         <v>239</v>
       </c>
@@ -20015,11 +20017,11 @@
         <v>1.35550089182616</v>
       </c>
       <c r="I263">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1752430799252876E-3</v>
       </c>
     </row>
-    <row r="264" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:9" ht="42.75">
       <c r="A264" s="1" t="s">
         <v>240</v>
       </c>
@@ -20045,11 +20047,11 @@
         <v>1.35680701343988</v>
       </c>
       <c r="I264">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.5659245014747361E-3</v>
       </c>
     </row>
-    <row r="265" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:9" ht="42.75">
       <c r="A265" s="1" t="s">
         <v>241</v>
       </c>
@@ -20075,11 +20077,11 @@
         <v>1.3556933496622401</v>
       </c>
       <c r="I265">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.9415930758125439E-3</v>
       </c>
     </row>
-    <row r="266" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:9" ht="42.75">
       <c r="A266" s="1" t="s">
         <v>242</v>
       </c>
@@ -20105,11 +20107,11 @@
         <v>1.3554609217195099</v>
       </c>
       <c r="I266">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.5628764987721512E-3</v>
       </c>
     </row>
-    <row r="267" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:9" ht="42.75">
       <c r="A267" s="1" t="s">
         <v>243</v>
       </c>
@@ -20135,11 +20137,11 @@
         <v>1.3611060715916099</v>
       </c>
       <c r="I267">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.3142877871552706E-3</v>
       </c>
     </row>
-    <row r="268" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:9" ht="42.75">
       <c r="A268" s="1" t="s">
         <v>244</v>
       </c>
@@ -20165,11 +20167,11 @@
         <v>1.35991177591153</v>
       </c>
       <c r="I268">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.080930567316596E-3</v>
       </c>
     </row>
-    <row r="269" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:9" ht="42.75">
       <c r="A269" s="1" t="s">
         <v>245</v>
       </c>
@@ -20195,11 +20197,11 @@
         <v>1.3607645407295701</v>
       </c>
       <c r="I269">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.086981741108657E-3</v>
       </c>
     </row>
-    <row r="270" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:9" ht="42.75">
       <c r="A270" s="1" t="s">
         <v>246</v>
       </c>
@@ -20225,11 +20227,11 @@
         <v>1.3654685189158899</v>
       </c>
       <c r="I270">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.468252943311888E-3</v>
       </c>
     </row>
-    <row r="271" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:9" ht="42.75">
       <c r="A271" s="1" t="s">
         <v>247</v>
       </c>
@@ -20255,11 +20257,11 @@
         <v>1.3672657381228599</v>
       </c>
       <c r="I271">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.0229456020168344E-3</v>
       </c>
     </row>
-    <row r="272" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:9" ht="42.75">
       <c r="A272" s="1" t="s">
         <v>248</v>
       </c>
@@ -20285,11 +20287,11 @@
         <v>1.36428049976999</v>
       </c>
       <c r="I272">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.6246644541519791E-3</v>
       </c>
     </row>
-    <row r="273" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:9" ht="42.75">
       <c r="A273" s="1" t="s">
         <v>249</v>
       </c>
@@ -20315,11 +20317,11 @@
         <v>1.36939615707218</v>
       </c>
       <c r="I273">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.8837425349856967E-3</v>
       </c>
     </row>
-    <row r="274" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:9" ht="42.75">
       <c r="A274" s="1" t="s">
         <v>250</v>
       </c>
@@ -20345,11 +20347,11 @@
         <v>1.3668714982338499</v>
       </c>
       <c r="I274">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.0399538471929258E-3</v>
       </c>
     </row>
-    <row r="275" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:9" ht="42.75">
       <c r="A275" s="1" t="s">
         <v>251</v>
       </c>
@@ -20375,11 +20377,11 @@
         <v>1.3662114192681001</v>
       </c>
       <c r="I275">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.5775531102099048E-3</v>
       </c>
     </row>
-    <row r="276" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:9" ht="42.75">
       <c r="A276" s="1" t="s">
         <v>252</v>
       </c>
@@ -20405,11 +20407,11 @@
         <v>1.3646550452370101</v>
       </c>
       <c r="I276">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1991173284969883E-3</v>
       </c>
     </row>
-    <row r="277" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:9" ht="42.75">
       <c r="A277" s="1" t="s">
         <v>253</v>
       </c>
@@ -20435,11 +20437,11 @@
         <v>1.3634665515115301</v>
       </c>
       <c r="I277">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>4.1231632087655725E-3</v>
       </c>
     </row>
-    <row r="278" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:9" ht="42.75">
       <c r="A278" s="1" t="s">
         <v>254</v>
       </c>
@@ -20465,11 +20467,11 @@
         <v>1.3567920177930901</v>
       </c>
       <c r="I278">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.4057085646243494E-3</v>
       </c>
     </row>
-    <row r="279" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:9" ht="42.75">
       <c r="A279" s="1" t="s">
         <v>255</v>
       </c>
@@ -20495,11 +20497,11 @@
         <v>1.35649907366866</v>
       </c>
       <c r="I279">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.479279235008851E-3</v>
       </c>
     </row>
-    <row r="280" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:9" ht="42.75">
       <c r="A280" s="1" t="s">
         <v>256</v>
       </c>
@@ -20525,11 +20527,11 @@
         <v>1.35141035366492</v>
       </c>
       <c r="I280">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>4.0962591885140859E-3</v>
       </c>
     </row>
-    <row r="281" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:9" ht="42.75">
       <c r="A281" s="1" t="s">
         <v>257</v>
       </c>
@@ -20555,11 +20557,11 @@
         <v>1.35438928583693</v>
       </c>
       <c r="I281">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>4.0874728576909859E-3</v>
       </c>
     </row>
-    <row r="282" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:9" ht="42.75">
       <c r="A282" s="1" t="s">
         <v>258</v>
       </c>
@@ -20585,11 +20587,11 @@
         <v>1.35019553306989</v>
       </c>
       <c r="I282">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.3341940954636777E-3</v>
       </c>
     </row>
-    <row r="283" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:9" ht="42.75">
       <c r="A283" s="1" t="s">
         <v>259</v>
       </c>
@@ -20615,11 +20617,11 @@
         <v>1.3524204518407701</v>
       </c>
       <c r="I283">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.7209903173989365E-3</v>
       </c>
     </row>
-    <row r="284" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:9" ht="42.75">
       <c r="A284" s="1" t="s">
         <v>260</v>
       </c>
@@ -20645,11 +20647,11 @@
         <v>1.35965040607513</v>
       </c>
       <c r="I284">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>4.6780955504835218E-3</v>
       </c>
     </row>
-    <row r="285" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:9" ht="42.75">
       <c r="A285" s="1" t="s">
         <v>261</v>
       </c>
@@ -20675,11 +20677,11 @@
         <v>1.3684384055624299</v>
       </c>
       <c r="I285">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>4.3615356091261138E-3</v>
       </c>
     </row>
-    <row r="286" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:9" ht="42.75">
       <c r="A286" s="1" t="s">
         <v>262</v>
       </c>
@@ -20705,11 +20707,11 @@
         <v>1.35651473501414</v>
       </c>
       <c r="I286">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>4.2271907331253925E-3</v>
       </c>
     </row>
-    <row r="287" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:9" ht="42.75">
       <c r="A287" s="1" t="s">
         <v>263</v>
       </c>
@@ -20735,11 +20737,11 @@
         <v>1.36522227052874</v>
       </c>
       <c r="I287">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.4753101947992944E-3</v>
       </c>
     </row>
-    <row r="288" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:9" ht="42.75">
       <c r="A288" s="1" t="s">
         <v>264</v>
       </c>
@@ -20765,11 +20767,11 @@
         <v>1.36782571532579</v>
       </c>
       <c r="I288">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.7626563678169293E-3</v>
       </c>
     </row>
-    <row r="289" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:9" ht="42.75">
       <c r="A289" s="1" t="s">
         <v>265</v>
       </c>
@@ -20795,11 +20797,11 @@
         <v>1.36802950154961</v>
       </c>
       <c r="I289">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1476349917578263E-3</v>
       </c>
     </row>
-    <row r="290" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:9" ht="42.75">
       <c r="A290" s="1" t="s">
         <v>266</v>
       </c>
@@ -20825,11 +20827,11 @@
         <v>1.3630234529095899</v>
       </c>
       <c r="I290">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.7221691623789189E-3</v>
       </c>
     </row>
-    <row r="291" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:9" ht="42.75">
       <c r="A291" s="1" t="s">
         <v>267</v>
       </c>
@@ -20855,11 +20857,11 @@
         <v>1.36702797096413</v>
       </c>
       <c r="I291">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.7138515154685274E-3</v>
       </c>
     </row>
-    <row r="292" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:9" ht="42.75">
       <c r="A292" s="1" t="s">
         <v>268</v>
       </c>
@@ -20885,11 +20887,11 @@
         <v>1.3662286539353801</v>
       </c>
       <c r="I292">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.9713595346613402E-3</v>
       </c>
     </row>
-    <row r="293" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:9" ht="42.75">
       <c r="A293" s="1" t="s">
         <v>269</v>
       </c>
@@ -20915,11 +20917,11 @@
         <v>1.3653126927192201</v>
       </c>
       <c r="I293">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1179510605047586E-3</v>
       </c>
     </row>
-    <row r="294" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:9" ht="42.75">
       <c r="A294" s="1" t="s">
         <v>270</v>
       </c>
@@ -20945,11 +20947,11 @@
         <v>1.36675467689598</v>
       </c>
       <c r="I294">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.3834128826894534E-3</v>
       </c>
     </row>
-    <row r="295" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:9" ht="42.75">
       <c r="A295" s="1" t="s">
         <v>271</v>
       </c>
@@ -20975,11 +20977,11 @@
         <v>1.3645146959369601</v>
       </c>
       <c r="I295">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.9514391245968369E-3</v>
       </c>
     </row>
-    <row r="296" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:9" ht="42.75">
       <c r="A296" s="1" t="s">
         <v>272</v>
       </c>
@@ -21005,11 +21007,11 @@
         <v>1.3650274749650799</v>
       </c>
       <c r="I296">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.8657085916863985E-3</v>
       </c>
     </row>
-    <row r="297" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:9" ht="42.75">
       <c r="A297" s="1" t="s">
         <v>273</v>
       </c>
@@ -21035,11 +21037,11 @@
         <v>1.3656274497946901</v>
       </c>
       <c r="I297">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.0004205231841199E-3</v>
       </c>
     </row>
-    <row r="298" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:9" ht="42.75">
       <c r="A298" s="1" t="s">
         <v>274</v>
       </c>
@@ -21065,11 +21067,11 @@
         <v>1.3662545861395201</v>
       </c>
       <c r="I298">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.4385565529818779E-3</v>
       </c>
     </row>
-    <row r="299" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:9" ht="42.75">
       <c r="A299" s="1" t="s">
         <v>275</v>
       </c>
@@ -21095,11 +21097,11 @@
         <v>1.36613317608998</v>
       </c>
       <c r="I299">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.8979336502672811E-3</v>
       </c>
     </row>
-    <row r="300" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:9" ht="42.75">
       <c r="A300" s="1" t="s">
         <v>276</v>
       </c>
@@ -21125,11 +21127,11 @@
         <v>1.3640842381865099</v>
       </c>
       <c r="I300">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.7750146265812306E-3</v>
       </c>
     </row>
-    <row r="301" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:9" ht="42.75">
       <c r="A301" s="1" t="s">
         <v>277</v>
       </c>
@@ -21155,11 +21157,11 @@
         <v>1.3680351664949699</v>
       </c>
       <c r="I301">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.599229067474717E-3</v>
       </c>
     </row>
-    <row r="302" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="302" spans="1:9" ht="42.75">
       <c r="A302" s="1" t="s">
         <v>278</v>
       </c>
@@ -21185,11 +21187,11 @@
         <v>1.36560087585368</v>
       </c>
       <c r="I302">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1184794761352332E-3</v>
       </c>
     </row>
-    <row r="303" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="303" spans="1:9" ht="42.75">
       <c r="A303" s="1" t="s">
         <v>279</v>
       </c>
@@ -21215,11 +21217,11 @@
         <v>1.36709325123165</v>
       </c>
       <c r="I303">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1448997014747776E-3</v>
       </c>
     </row>
-    <row r="304" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="304" spans="1:9" ht="42.75">
       <c r="A304" s="1" t="s">
         <v>280</v>
       </c>
@@ -21245,11 +21247,11 @@
         <v>1.3651668180998899</v>
       </c>
       <c r="I304">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.7859891431840952E-3</v>
       </c>
     </row>
-    <row r="305" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="305" spans="1:9" ht="42.75">
       <c r="A305" s="1" t="s">
         <v>281</v>
       </c>
@@ -21275,11 +21277,11 @@
         <v>1.3653415861354801</v>
       </c>
       <c r="I305">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.9952984407034216E-3</v>
       </c>
     </row>
-    <row r="306" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="306" spans="1:9" ht="42.75">
       <c r="A306" s="1" t="s">
         <v>282</v>
       </c>
@@ -21305,11 +21307,11 @@
         <v>1.3643861435771201</v>
       </c>
       <c r="I306">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>2.8646795553659149E-3</v>
       </c>
     </row>
-    <row r="307" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="307" spans="1:9" ht="42.75">
       <c r="A307" s="1" t="s">
         <v>283</v>
       </c>
@@ -21335,11 +21337,11 @@
         <v>1.3636598487009499</v>
       </c>
       <c r="I307">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.1031680899929414E-3</v>
       </c>
     </row>
-    <row r="308" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="308" spans="1:9" ht="42.75">
       <c r="A308" s="1" t="s">
         <v>284</v>
       </c>
@@ -21365,7 +21367,7 @@
         <v>1.3572073321533</v>
       </c>
       <c r="I308">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>3.4551547307947162E-3</v>
       </c>
     </row>

</xml_diff>